<commit_message>
Add completion statements, property purchase analysis and draft P&L / balance sheet for Alino Property Ltd
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UszXj8jDKmjemVNstTQPa2
</commit_message>
<xml_diff>
--- a/data/Monzo_Reconciliation.xlsx
+++ b/data/Monzo_Reconciliation.xlsx
@@ -11,8 +11,11 @@
     <sheet name="Monzo Reconciliation" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Monzo Transactions" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="Monzo Categories" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="Completion Lines" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="Property Purchase" sheetId="5" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
+    <definedName function="false" hidden="true" localSheetId="3" name="_xlnm._FilterDatabase" vbProcedure="false">'Completion Lines'!$A$1:$G$41</definedName>
     <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Monzo Transactions'!$A$1:$N$37</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
@@ -92,8 +95,30 @@
 </comments>
 </file>
 
+<file path=xl/comments4.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <authors>
+    <author>Unknown Author</author>
+  </authors>
+  <commentList>
+    <comment ref="G1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">My accounting classification. Edit freely – Property Purchase sheet uses SUMIFS on this column.</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="290" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="473" uniqueCount="201">
   <si>
     <t xml:space="preserve">Monzo Business Account (Alino Property Ltd) – Monthly Reconciliation</t>
   </si>
@@ -399,17 +424,315 @@
   </si>
   <si>
     <t xml:space="preserve">Check vs reconciliation (should be 0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Statement</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Item</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Paid In (£)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Paid Out – net (£)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VAT (£)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Paid Out – gross (£)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Classification</t>
+  </si>
+  <si>
+    <t xml:space="preserve">30 Strensall Rd – Remortgage (17/07/2025)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mortgage advance minus 3rd party solicitors fee</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Funding – Strensall remortgage advance (net)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Money on account 8.4.2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Funding – money on account</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Legal Fees</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Finance cost – Strensall remortgage</t>
+  </si>
+  <si>
+    <t xml:space="preserve">File Setup Fee</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mortgage Fee</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Third party sols fee for dealing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No Searches Indemnity Insurance Policy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Land Charges Search (£6 per person) x 3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bank Transfer Fee</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Land Registry Documents</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Land Registry Search – OS1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Land Registry Fees</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MR01 Companies House registration of charge</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Company winding up search</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Company search – Global</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Balance due on completion → sent to Cairnsford purchase</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Transfer – Strensall proceeds to Cairnsford</t>
+  </si>
+  <si>
+    <t xml:space="preserve">36 Cairnsford Rd – Purchase (17/07/2025)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Purchase Price</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Property cost – purchase price</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Money on Account</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mortgage advance from lender's solicitors (net of their fees)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Funding – Together Commercial mortgage (net)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Proceeds from 30 Strensall</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Money from client – Alvine 14.7.25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Funding – Alvine Tchega</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Money from client – Kakmeni 14.7.25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Funding – Kakmeni</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Property cost – legal &amp; acquisition fees</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mortgage Admin Fee</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Finance cost – Cairnsford mortgage</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stamp Duty Land Tax Form Fee</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Anti-Money Laundering Check Fee (£30 pp)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Third party lender solicitors fee</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Policy arrangement fee</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Land Registry Search</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Land Charges Search (£6 pp)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Searches Pack</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stamp Duty (SDLT)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Property cost – Stamp Duty (SDLT)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Search perusal Fee</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Company search fee</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MR01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Winding up Search Fee</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Insolvency indemnity policy required by lender</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Check against statement totals</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Paid In – calc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Paid In – statement</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Paid Out – calc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Paid Out – statement</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PDF: CompletionStatement_1093081_Tchega_2025-07-15 (total out £1,670 + balance due £131,958)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PDF: Complation_Statement (DWS Legal), totals £500,658.94 / £500,658.94, balance £0.00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">36 Cairnsford Road, Leicester LE2 6GF – Purchase Analysis (Alino Property Ltd)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Completed 17/07/2025, funded partly by remortgage of 30 Strensall Road. All figures are SUMIFS over Completion Lines (gross incl. VAT – treated as irrecoverable).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A. Cost of property (capitalise – fixed asset / investment property)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">£</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Purchase price</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stamp Duty Land Tax</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SDLT is part of the cost of the property</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Legal &amp; acquisition fees (incl. VAT)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Legal, searches, Land Registry, AML, SDLT form, bank transfer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total cost of 36 Cairnsford Road</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B. Finance / loan arrangement costs (not property cost)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cairnsford mortgage – lender-related fees</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mortgage admin, lender sols, policy arrangement, insolvency indemnity, MR01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">30 Strensall remortgage – all costs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Whole remortgage statement (£1,670); spread over loan term or expense</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total finance costs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C. How the purchase was funded (Cairnsford statement – paid in)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Together Commercial mortgage (net advance)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Net of lender's solicitor fees; gross loan not shown on statement</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Proceeds of 30 Strensall remortgage</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Equals £133,528 advance + £100 on account − £1,670 costs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alvine Tchega – money in 14/07/2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Director's loan to company (confirm)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kakmeni – money in 14/07/2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Loan or investment? Ties to Kakmeni receipts on Monzo (confirm)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Money on account (Cairnsford)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total funds in for purchase</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D. Check</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cost (A) + Cairnsford finance fees</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Funds in (C)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Difference (should be 0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">E. Ongoing mortgage payments (from Monzo business account)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Together Commercial DD 10395974-002 – paid Oct-25 to Feb-26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Likely the larger Cairnsford loan (confirm with Together)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Together Commercial DD 10395973-002 – paid Oct-25 to Feb-26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Likely the 30 Strensall remortgage (confirm with Together)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="\£#,##0.00;&quot;-£&quot;#,##0.00;\-"/>
     <numFmt numFmtId="166" formatCode="dd/mm/yyyy"/>
     <numFmt numFmtId="167" formatCode="0"/>
+    <numFmt numFmtId="168" formatCode="\£#,##0.00;&quot;-£&quot;#,##0.00;\-"/>
   </numFmts>
   <fonts count="12">
     <font>
@@ -553,7 +876,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="36">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -639,6 +962,62 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -748,6 +1127,10 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
 </file>
 
@@ -3642,4 +4025,1384 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:G46"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="55"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="44"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="22" t="s">
+        <v>109</v>
+      </c>
+      <c r="B2" s="22" t="s">
+        <v>110</v>
+      </c>
+      <c r="C2" s="23" t="n">
+        <v>133528</v>
+      </c>
+      <c r="D2" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" s="24" t="n">
+        <f aca="false">D2+E2</f>
+        <v>0</v>
+      </c>
+      <c r="G2" s="22" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="22" t="s">
+        <v>109</v>
+      </c>
+      <c r="B3" s="22" t="s">
+        <v>112</v>
+      </c>
+      <c r="C3" s="23" t="n">
+        <v>100</v>
+      </c>
+      <c r="D3" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" s="24" t="n">
+        <f aca="false">D3+E3</f>
+        <v>0</v>
+      </c>
+      <c r="G3" s="22" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="22" t="s">
+        <v>109</v>
+      </c>
+      <c r="B4" s="22" t="s">
+        <v>114</v>
+      </c>
+      <c r="C4" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" s="23" t="n">
+        <v>650</v>
+      </c>
+      <c r="E4" s="23" t="n">
+        <v>130</v>
+      </c>
+      <c r="F4" s="24" t="n">
+        <f aca="false">D4+E4</f>
+        <v>780</v>
+      </c>
+      <c r="G4" s="22" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="22" t="s">
+        <v>109</v>
+      </c>
+      <c r="B5" s="22" t="s">
+        <v>116</v>
+      </c>
+      <c r="C5" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" s="23" t="n">
+        <v>35</v>
+      </c>
+      <c r="E5" s="23" t="n">
+        <v>7</v>
+      </c>
+      <c r="F5" s="24" t="n">
+        <f aca="false">D5+E5</f>
+        <v>42</v>
+      </c>
+      <c r="G5" s="22" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="22" t="s">
+        <v>109</v>
+      </c>
+      <c r="B6" s="22" t="s">
+        <v>117</v>
+      </c>
+      <c r="C6" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" s="23" t="n">
+        <v>200</v>
+      </c>
+      <c r="E6" s="23" t="n">
+        <v>40</v>
+      </c>
+      <c r="F6" s="24" t="n">
+        <f aca="false">D6+E6</f>
+        <v>240</v>
+      </c>
+      <c r="G6" s="22" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="22" t="s">
+        <v>109</v>
+      </c>
+      <c r="B7" s="22" t="s">
+        <v>118</v>
+      </c>
+      <c r="C7" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" s="23" t="n">
+        <v>300</v>
+      </c>
+      <c r="E7" s="23" t="n">
+        <v>60</v>
+      </c>
+      <c r="F7" s="24" t="n">
+        <f aca="false">D7+E7</f>
+        <v>360</v>
+      </c>
+      <c r="G7" s="22" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="22" t="s">
+        <v>109</v>
+      </c>
+      <c r="B8" s="22" t="s">
+        <v>119</v>
+      </c>
+      <c r="C8" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" s="23" t="n">
+        <v>29</v>
+      </c>
+      <c r="E8" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" s="24" t="n">
+        <f aca="false">D8+E8</f>
+        <v>29</v>
+      </c>
+      <c r="G8" s="22" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="22" t="s">
+        <v>109</v>
+      </c>
+      <c r="B9" s="22" t="s">
+        <v>120</v>
+      </c>
+      <c r="C9" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" s="23" t="n">
+        <v>18</v>
+      </c>
+      <c r="E9" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" s="24" t="n">
+        <f aca="false">D9+E9</f>
+        <v>18</v>
+      </c>
+      <c r="G9" s="22" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="22" t="s">
+        <v>109</v>
+      </c>
+      <c r="B10" s="22" t="s">
+        <v>121</v>
+      </c>
+      <c r="C10" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" s="23" t="n">
+        <v>45</v>
+      </c>
+      <c r="E10" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" s="24" t="n">
+        <f aca="false">D10+E10</f>
+        <v>45</v>
+      </c>
+      <c r="G10" s="22" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="22" t="s">
+        <v>109</v>
+      </c>
+      <c r="B11" s="22" t="s">
+        <v>122</v>
+      </c>
+      <c r="C11" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" s="23" t="n">
+        <v>14</v>
+      </c>
+      <c r="E11" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" s="24" t="n">
+        <f aca="false">D11+E11</f>
+        <v>14</v>
+      </c>
+      <c r="G11" s="22" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="22" t="s">
+        <v>109</v>
+      </c>
+      <c r="B12" s="22" t="s">
+        <v>123</v>
+      </c>
+      <c r="C12" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" s="23" t="n">
+        <v>7</v>
+      </c>
+      <c r="E12" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" s="24" t="n">
+        <f aca="false">D12+E12</f>
+        <v>7</v>
+      </c>
+      <c r="G12" s="22" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="22" t="s">
+        <v>109</v>
+      </c>
+      <c r="B13" s="22" t="s">
+        <v>124</v>
+      </c>
+      <c r="C13" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" s="23" t="n">
+        <v>45</v>
+      </c>
+      <c r="E13" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" s="24" t="n">
+        <f aca="false">D13+E13</f>
+        <v>45</v>
+      </c>
+      <c r="G13" s="22" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="22" t="s">
+        <v>109</v>
+      </c>
+      <c r="B14" s="22" t="s">
+        <v>125</v>
+      </c>
+      <c r="C14" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" s="23" t="n">
+        <v>15</v>
+      </c>
+      <c r="E14" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" s="24" t="n">
+        <f aca="false">D14+E14</f>
+        <v>15</v>
+      </c>
+      <c r="G14" s="22" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="22" t="s">
+        <v>109</v>
+      </c>
+      <c r="B15" s="22" t="s">
+        <v>126</v>
+      </c>
+      <c r="C15" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D15" s="23" t="n">
+        <v>15</v>
+      </c>
+      <c r="E15" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="24" t="n">
+        <f aca="false">D15+E15</f>
+        <v>15</v>
+      </c>
+      <c r="G15" s="22" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="22" t="s">
+        <v>109</v>
+      </c>
+      <c r="B16" s="22" t="s">
+        <v>127</v>
+      </c>
+      <c r="C16" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D16" s="23" t="n">
+        <v>60</v>
+      </c>
+      <c r="E16" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" s="24" t="n">
+        <f aca="false">D16+E16</f>
+        <v>60</v>
+      </c>
+      <c r="G16" s="22" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="22" t="s">
+        <v>109</v>
+      </c>
+      <c r="B17" s="22" t="s">
+        <v>128</v>
+      </c>
+      <c r="C17" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" s="23" t="n">
+        <v>131958</v>
+      </c>
+      <c r="E17" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" s="24" t="n">
+        <f aca="false">D17+E17</f>
+        <v>131958</v>
+      </c>
+      <c r="G17" s="22" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="22" t="s">
+        <v>130</v>
+      </c>
+      <c r="B18" s="22" t="s">
+        <v>131</v>
+      </c>
+      <c r="C18" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D18" s="23" t="n">
+        <v>462000</v>
+      </c>
+      <c r="E18" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" s="24" t="n">
+        <f aca="false">D18+E18</f>
+        <v>462000</v>
+      </c>
+      <c r="G18" s="22" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="22" t="s">
+        <v>130</v>
+      </c>
+      <c r="B19" s="22" t="s">
+        <v>133</v>
+      </c>
+      <c r="C19" s="23" t="n">
+        <v>400</v>
+      </c>
+      <c r="D19" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" s="24" t="n">
+        <f aca="false">D19+E19</f>
+        <v>0</v>
+      </c>
+      <c r="G19" s="22" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="22" t="s">
+        <v>130</v>
+      </c>
+      <c r="B20" s="22" t="s">
+        <v>134</v>
+      </c>
+      <c r="C20" s="23" t="n">
+        <v>311938.6</v>
+      </c>
+      <c r="D20" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="E20" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" s="24" t="n">
+        <f aca="false">D20+E20</f>
+        <v>0</v>
+      </c>
+      <c r="G20" s="22" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="22" t="s">
+        <v>130</v>
+      </c>
+      <c r="B21" s="22" t="s">
+        <v>136</v>
+      </c>
+      <c r="C21" s="23" t="n">
+        <v>131958</v>
+      </c>
+      <c r="D21" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="E21" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" s="24" t="n">
+        <f aca="false">D21+E21</f>
+        <v>0</v>
+      </c>
+      <c r="G21" s="22" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="22" t="s">
+        <v>130</v>
+      </c>
+      <c r="B22" s="22" t="s">
+        <v>137</v>
+      </c>
+      <c r="C22" s="23" t="n">
+        <v>18362.34</v>
+      </c>
+      <c r="D22" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="E22" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="F22" s="24" t="n">
+        <f aca="false">D22+E22</f>
+        <v>0</v>
+      </c>
+      <c r="G22" s="22" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="22" t="s">
+        <v>130</v>
+      </c>
+      <c r="B23" s="22" t="s">
+        <v>139</v>
+      </c>
+      <c r="C23" s="23" t="n">
+        <v>38000</v>
+      </c>
+      <c r="D23" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="E23" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="F23" s="24" t="n">
+        <f aca="false">D23+E23</f>
+        <v>0</v>
+      </c>
+      <c r="G23" s="22" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="22" t="s">
+        <v>130</v>
+      </c>
+      <c r="B24" s="22" t="s">
+        <v>114</v>
+      </c>
+      <c r="C24" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D24" s="23" t="n">
+        <v>775</v>
+      </c>
+      <c r="E24" s="23" t="n">
+        <v>155</v>
+      </c>
+      <c r="F24" s="24" t="n">
+        <f aca="false">D24+E24</f>
+        <v>930</v>
+      </c>
+      <c r="G24" s="22" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="22" t="s">
+        <v>130</v>
+      </c>
+      <c r="B25" s="22" t="s">
+        <v>142</v>
+      </c>
+      <c r="C25" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D25" s="23" t="n">
+        <v>100</v>
+      </c>
+      <c r="E25" s="23" t="n">
+        <v>20</v>
+      </c>
+      <c r="F25" s="24" t="n">
+        <f aca="false">D25+E25</f>
+        <v>120</v>
+      </c>
+      <c r="G25" s="22" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="22" t="s">
+        <v>130</v>
+      </c>
+      <c r="B26" s="22" t="s">
+        <v>116</v>
+      </c>
+      <c r="C26" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D26" s="23" t="n">
+        <v>35</v>
+      </c>
+      <c r="E26" s="23" t="n">
+        <v>7</v>
+      </c>
+      <c r="F26" s="24" t="n">
+        <f aca="false">D26+E26</f>
+        <v>42</v>
+      </c>
+      <c r="G26" s="22" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="22" t="s">
+        <v>130</v>
+      </c>
+      <c r="B27" s="22" t="s">
+        <v>144</v>
+      </c>
+      <c r="C27" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D27" s="23" t="n">
+        <v>75</v>
+      </c>
+      <c r="E27" s="23" t="n">
+        <v>15</v>
+      </c>
+      <c r="F27" s="24" t="n">
+        <f aca="false">D27+E27</f>
+        <v>90</v>
+      </c>
+      <c r="G27" s="22" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="22" t="s">
+        <v>130</v>
+      </c>
+      <c r="B28" s="22" t="s">
+        <v>145</v>
+      </c>
+      <c r="C28" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D28" s="23" t="n">
+        <v>60</v>
+      </c>
+      <c r="E28" s="23" t="n">
+        <v>12</v>
+      </c>
+      <c r="F28" s="24" t="n">
+        <f aca="false">D28+E28</f>
+        <v>72</v>
+      </c>
+      <c r="G28" s="22" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="22" t="s">
+        <v>130</v>
+      </c>
+      <c r="B29" s="22" t="s">
+        <v>146</v>
+      </c>
+      <c r="C29" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D29" s="23" t="n">
+        <v>300</v>
+      </c>
+      <c r="E29" s="23" t="n">
+        <v>60</v>
+      </c>
+      <c r="F29" s="24" t="n">
+        <f aca="false">D29+E29</f>
+        <v>360</v>
+      </c>
+      <c r="G29" s="22" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="22" t="s">
+        <v>130</v>
+      </c>
+      <c r="B30" s="22" t="s">
+        <v>147</v>
+      </c>
+      <c r="C30" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D30" s="23" t="n">
+        <v>50</v>
+      </c>
+      <c r="E30" s="23" t="n">
+        <v>10</v>
+      </c>
+      <c r="F30" s="24" t="n">
+        <f aca="false">D30+E30</f>
+        <v>60</v>
+      </c>
+      <c r="G30" s="22" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="22" t="s">
+        <v>130</v>
+      </c>
+      <c r="B31" s="22" t="s">
+        <v>148</v>
+      </c>
+      <c r="C31" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D31" s="23" t="n">
+        <v>7</v>
+      </c>
+      <c r="E31" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="F31" s="24" t="n">
+        <f aca="false">D31+E31</f>
+        <v>7</v>
+      </c>
+      <c r="G31" s="22" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="22" t="s">
+        <v>130</v>
+      </c>
+      <c r="B32" s="22" t="s">
+        <v>149</v>
+      </c>
+      <c r="C32" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D32" s="23" t="n">
+        <v>18</v>
+      </c>
+      <c r="E32" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="F32" s="24" t="n">
+        <f aca="false">D32+E32</f>
+        <v>18</v>
+      </c>
+      <c r="G32" s="22" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="22" t="s">
+        <v>130</v>
+      </c>
+      <c r="B33" s="22" t="s">
+        <v>121</v>
+      </c>
+      <c r="C33" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D33" s="23" t="n">
+        <v>45</v>
+      </c>
+      <c r="E33" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="F33" s="24" t="n">
+        <f aca="false">D33+E33</f>
+        <v>45</v>
+      </c>
+      <c r="G33" s="22" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="22" t="s">
+        <v>130</v>
+      </c>
+      <c r="B34" s="22" t="s">
+        <v>150</v>
+      </c>
+      <c r="C34" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D34" s="23" t="n">
+        <v>109.66</v>
+      </c>
+      <c r="E34" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="F34" s="24" t="n">
+        <f aca="false">D34+E34</f>
+        <v>109.66</v>
+      </c>
+      <c r="G34" s="22" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="22" t="s">
+        <v>130</v>
+      </c>
+      <c r="B35" s="22" t="s">
+        <v>124</v>
+      </c>
+      <c r="C35" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D35" s="23" t="n">
+        <v>150</v>
+      </c>
+      <c r="E35" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="F35" s="24" t="n">
+        <f aca="false">D35+E35</f>
+        <v>150</v>
+      </c>
+      <c r="G35" s="22" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="22" t="s">
+        <v>130</v>
+      </c>
+      <c r="B36" s="22" t="s">
+        <v>151</v>
+      </c>
+      <c r="C36" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D36" s="23" t="n">
+        <v>36200</v>
+      </c>
+      <c r="E36" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="F36" s="24" t="n">
+        <f aca="false">D36+E36</f>
+        <v>36200</v>
+      </c>
+      <c r="G36" s="22" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="22" t="s">
+        <v>130</v>
+      </c>
+      <c r="B37" s="22" t="s">
+        <v>153</v>
+      </c>
+      <c r="C37" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D37" s="23" t="n">
+        <v>200.28</v>
+      </c>
+      <c r="E37" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="F37" s="24" t="n">
+        <f aca="false">D37+E37</f>
+        <v>200.28</v>
+      </c>
+      <c r="G37" s="22" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="22" t="s">
+        <v>130</v>
+      </c>
+      <c r="B38" s="22" t="s">
+        <v>154</v>
+      </c>
+      <c r="C38" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D38" s="23" t="n">
+        <v>60</v>
+      </c>
+      <c r="E38" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="F38" s="24" t="n">
+        <f aca="false">D38+E38</f>
+        <v>60</v>
+      </c>
+      <c r="G38" s="22" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="22" t="s">
+        <v>130</v>
+      </c>
+      <c r="B39" s="22" t="s">
+        <v>155</v>
+      </c>
+      <c r="C39" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D39" s="23" t="n">
+        <v>15</v>
+      </c>
+      <c r="E39" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="F39" s="24" t="n">
+        <f aca="false">D39+E39</f>
+        <v>15</v>
+      </c>
+      <c r="G39" s="22" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="22" t="s">
+        <v>130</v>
+      </c>
+      <c r="B40" s="22" t="s">
+        <v>156</v>
+      </c>
+      <c r="C40" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D40" s="23" t="n">
+        <v>20</v>
+      </c>
+      <c r="E40" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="F40" s="24" t="n">
+        <f aca="false">D40+E40</f>
+        <v>20</v>
+      </c>
+      <c r="G40" s="22" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="22" t="s">
+        <v>130</v>
+      </c>
+      <c r="B41" s="22" t="s">
+        <v>157</v>
+      </c>
+      <c r="C41" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D41" s="23" t="n">
+        <v>160</v>
+      </c>
+      <c r="E41" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="F41" s="24" t="n">
+        <f aca="false">D41+E41</f>
+        <v>160</v>
+      </c>
+      <c r="G41" s="22" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="25" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="26" t="s">
+        <v>102</v>
+      </c>
+      <c r="B44" s="27"/>
+      <c r="C44" s="26" t="s">
+        <v>159</v>
+      </c>
+      <c r="D44" s="26" t="s">
+        <v>160</v>
+      </c>
+      <c r="E44" s="26" t="s">
+        <v>161</v>
+      </c>
+      <c r="F44" s="26" t="s">
+        <v>162</v>
+      </c>
+      <c r="G44" s="26" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="22" t="s">
+        <v>109</v>
+      </c>
+      <c r="B45" s="28" t="s">
+        <v>163</v>
+      </c>
+      <c r="C45" s="24" t="n">
+        <f aca="false">SUMIFS($C$2:$C$41,$A$2:$A$41,$A45)</f>
+        <v>133628</v>
+      </c>
+      <c r="D45" s="23" t="n">
+        <v>133628</v>
+      </c>
+      <c r="E45" s="24" t="n">
+        <f aca="false">SUMIFS($F$2:$F$41,$A$2:$A$41,$A45)</f>
+        <v>133628</v>
+      </c>
+      <c r="F45" s="23" t="n">
+        <v>133628</v>
+      </c>
+      <c r="G45" s="25" t="str">
+        <f aca="false">IF(AND(ROUND(C45-D45,2)=0,ROUND(E45-F45,2)=0,ROUND(C45-E45,2)=0),"Agrees – balances to £0","CHECK")</f>
+        <v>Agrees – balances to £0</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="22" t="s">
+        <v>130</v>
+      </c>
+      <c r="B46" s="28" t="s">
+        <v>164</v>
+      </c>
+      <c r="C46" s="24" t="n">
+        <f aca="false">SUMIFS($C$2:$C$41,$A$2:$A$41,$A46)</f>
+        <v>500658.94</v>
+      </c>
+      <c r="D46" s="23" t="n">
+        <v>500658.94</v>
+      </c>
+      <c r="E46" s="24" t="n">
+        <f aca="false">SUMIFS($F$2:$F$41,$A$2:$A$41,$A46)</f>
+        <v>500658.94</v>
+      </c>
+      <c r="F46" s="23" t="n">
+        <v>500658.94</v>
+      </c>
+      <c r="G46" s="25" t="str">
+        <f aca="false">IF(AND(ROUND(C46-D46,2)=0,ROUND(E46-F46,2)=0,ROUND(C46-E46,2)=0),"Agrees – balances to £0","CHECK")</f>
+        <v>Agrees – balances to £0</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:G41"/>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+  <drawing r:id="rId2"/>
+  <legacyDrawing r:id="rId3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:C30"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="75"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="29" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="28" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="26" t="s">
+        <v>167</v>
+      </c>
+      <c r="B4" s="26" t="s">
+        <v>168</v>
+      </c>
+      <c r="C4" s="26" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="30" t="s">
+        <v>169</v>
+      </c>
+      <c r="B5" s="31" t="n">
+        <f aca="false">SUMIFS('Completion Lines'!$F$2:$F$41,'Completion Lines'!$G$2:$G$41,"Property cost – purchase price")</f>
+        <v>462000</v>
+      </c>
+      <c r="C5" s="32"/>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="30" t="s">
+        <v>170</v>
+      </c>
+      <c r="B6" s="31" t="n">
+        <f aca="false">SUMIFS('Completion Lines'!$F$2:$F$41,'Completion Lines'!$G$2:$G$41,"Property cost – Stamp Duty (SDLT)")</f>
+        <v>36200</v>
+      </c>
+      <c r="C6" s="32" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="30" t="s">
+        <v>172</v>
+      </c>
+      <c r="B7" s="31" t="n">
+        <f aca="false">SUMIFS('Completion Lines'!$F$2:$F$41,'Completion Lines'!$G$2:$G$41,"Property cost – legal &amp; acquisition fees")</f>
+        <v>1743.94</v>
+      </c>
+      <c r="C7" s="32" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="33" t="s">
+        <v>174</v>
+      </c>
+      <c r="B8" s="34" t="n">
+        <f aca="false">SUM(B5:B7)</f>
+        <v>499943.94</v>
+      </c>
+      <c r="C8" s="33"/>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="26" t="s">
+        <v>175</v>
+      </c>
+      <c r="B10" s="26" t="s">
+        <v>168</v>
+      </c>
+      <c r="C10" s="26" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="30" t="s">
+        <v>176</v>
+      </c>
+      <c r="B11" s="31" t="n">
+        <f aca="false">SUMIFS('Completion Lines'!$F$2:$F$41,'Completion Lines'!$G$2:$G$41,"Finance cost – Cairnsford mortgage")</f>
+        <v>715</v>
+      </c>
+      <c r="C11" s="32" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="30" t="s">
+        <v>178</v>
+      </c>
+      <c r="B12" s="31" t="n">
+        <f aca="false">SUMIFS('Completion Lines'!$F$2:$F$41,'Completion Lines'!$G$2:$G$41,"Finance cost – Strensall remortgage")</f>
+        <v>1670</v>
+      </c>
+      <c r="C12" s="32" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="33" t="s">
+        <v>180</v>
+      </c>
+      <c r="B13" s="34" t="n">
+        <f aca="false">SUM(B11:B12)</f>
+        <v>2385</v>
+      </c>
+      <c r="C13" s="33"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="26" t="s">
+        <v>181</v>
+      </c>
+      <c r="B15" s="26" t="s">
+        <v>168</v>
+      </c>
+      <c r="C15" s="26" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="30" t="s">
+        <v>182</v>
+      </c>
+      <c r="B16" s="31" t="n">
+        <f aca="false">SUMIFS('Completion Lines'!$C$2:$C$41,'Completion Lines'!$G$2:$G$41,"Funding – Together Commercial mortgage (net)")</f>
+        <v>311938.6</v>
+      </c>
+      <c r="C16" s="32" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="30" t="s">
+        <v>184</v>
+      </c>
+      <c r="B17" s="31" t="n">
+        <f aca="false">SUMIFS('Completion Lines'!$C$2:$C$41,'Completion Lines'!$G$2:$G$41,"Transfer – Strensall proceeds to Cairnsford",'Completion Lines'!$A$2:$A$41,"36 Cairnsford Rd – Purchase (17/07/2025)")</f>
+        <v>131958</v>
+      </c>
+      <c r="C17" s="32" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="30" t="s">
+        <v>186</v>
+      </c>
+      <c r="B18" s="31" t="n">
+        <f aca="false">SUMIFS('Completion Lines'!$C$2:$C$41,'Completion Lines'!$G$2:$G$41,"Funding – Alvine Tchega")</f>
+        <v>18362.34</v>
+      </c>
+      <c r="C18" s="32" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="30" t="s">
+        <v>188</v>
+      </c>
+      <c r="B19" s="31" t="n">
+        <f aca="false">SUMIFS('Completion Lines'!$C$2:$C$41,'Completion Lines'!$G$2:$G$41,"Funding – Kakmeni")</f>
+        <v>38000</v>
+      </c>
+      <c r="C19" s="32" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="30" t="s">
+        <v>190</v>
+      </c>
+      <c r="B20" s="31" t="n">
+        <f aca="false">SUMIFS('Completion Lines'!$C$2:$C$41,'Completion Lines'!$G$2:$G$41,"Funding – money on account",'Completion Lines'!$A$2:$A$41,"36 Cairnsford Rd – Purchase (17/07/2025)")</f>
+        <v>400</v>
+      </c>
+      <c r="C20" s="32"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="33" t="s">
+        <v>191</v>
+      </c>
+      <c r="B21" s="34" t="n">
+        <f aca="false">SUM(B16:B20)</f>
+        <v>500658.94</v>
+      </c>
+      <c r="C21" s="33"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="26" t="s">
+        <v>192</v>
+      </c>
+      <c r="B23" s="26" t="s">
+        <v>168</v>
+      </c>
+      <c r="C23" s="26" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="30" t="s">
+        <v>193</v>
+      </c>
+      <c r="B24" s="31" t="n">
+        <f aca="false">B8+B11</f>
+        <v>500658.94</v>
+      </c>
+      <c r="C24" s="32"/>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="30" t="s">
+        <v>194</v>
+      </c>
+      <c r="B25" s="31" t="n">
+        <f aca="false">B21</f>
+        <v>500658.94</v>
+      </c>
+      <c r="C25" s="32"/>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="25" t="s">
+        <v>195</v>
+      </c>
+      <c r="B26" s="35" t="n">
+        <f aca="false">ROUND(B24-B25,2)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="26" t="s">
+        <v>196</v>
+      </c>
+      <c r="B28" s="26" t="s">
+        <v>168</v>
+      </c>
+      <c r="C28" s="26" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="30" t="s">
+        <v>197</v>
+      </c>
+      <c r="B29" s="31" t="n">
+        <f aca="false">-SUMIFS('Monzo Transactions'!$J:$J,'Monzo Transactions'!$E:$E,"10395974-002")</f>
+        <v>10699.15</v>
+      </c>
+      <c r="C29" s="32" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="30" t="s">
+        <v>199</v>
+      </c>
+      <c r="B30" s="31" t="n">
+        <f aca="false">-SUMIFS('Monzo Transactions'!$J:$J,'Monzo Transactions'!$E:$E,"10395973-002")</f>
+        <v>5802.9</v>
+      </c>
+      <c r="C30" s="32" t="s">
+        <v>200</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>